<commit_message>
Section 1 and section 2 are done and closed after testing with multiple data
</commit_message>
<xml_diff>
--- a/automation_engine/modules/fla/excel/FLA_comparsion.xlsx
+++ b/automation_engine/modules/fla/excel/FLA_comparsion.xlsx
@@ -2060,7 +2060,7 @@
       <c r="C7" s="23" t="n"/>
       <c r="D7" s="188" t="inlineStr">
         <is>
-          <t>Previous FLA form, Unless company wants to change it.</t>
+          <t>PREVIOUS FLA</t>
         </is>
       </c>
     </row>
@@ -2078,7 +2078,7 @@
       <c r="C8" s="23" t="n"/>
       <c r="D8" s="188" t="inlineStr">
         <is>
-          <t>Previous FLA form, Unless company wants to change it.</t>
+          <t>PREVIOUS FLA - UNLESS THERE IS CHANGE</t>
         </is>
       </c>
     </row>
@@ -2096,7 +2096,7 @@
       <c r="C9" s="23" t="n"/>
       <c r="D9" s="188" t="inlineStr">
         <is>
-          <t>Previous FLA form, Unless company wants to change it.</t>
+          <t>PREVIOUS FLA</t>
         </is>
       </c>
     </row>
@@ -2128,7 +2128,7 @@
       <c r="C11" s="23" t="n"/>
       <c r="D11" s="188" t="inlineStr">
         <is>
-          <t>Previous FLA form, Unless company wants to change it.</t>
+          <t>PREVIOUS FLA - UNLESS THERE IS CHANGE</t>
         </is>
       </c>
     </row>
@@ -2146,7 +2146,7 @@
       <c r="C12" s="23" t="n"/>
       <c r="D12" s="188" t="inlineStr">
         <is>
-          <t>Previous FLA form, Unless company wants to change it.</t>
+          <t>PREVIOUS FLA</t>
         </is>
       </c>
     </row>
@@ -2164,7 +2164,7 @@
       <c r="C13" s="23" t="n"/>
       <c r="D13" s="188" t="inlineStr">
         <is>
-          <t>Previous FLA form, Unless company wants to change it.</t>
+          <t>PREVIOUS FLA</t>
         </is>
       </c>
     </row>
@@ -2203,9 +2203,7 @@
       <c r="C15" s="23" t="n"/>
       <c r="D15" s="188" t="inlineStr">
         <is>
-          <t>1) Previous FLA form, 
-2) Cross verify the highest revenue generating operation, if same, no problem.
-3) If different, to change it based on company verification</t>
+          <t>PREVIOUS FLA</t>
         </is>
       </c>
     </row>
@@ -2365,7 +2363,7 @@
       <c r="C26" s="192" t="n"/>
       <c r="D26" s="193" t="inlineStr">
         <is>
-          <t>FINANCIALS + LIST OF SHAREHOLDER</t>
+          <t>PREVIOUS FLA - UNLESS THERE IS CHANGE</t>
         </is>
       </c>
     </row>
@@ -2379,7 +2377,7 @@
       <c r="C27" s="192" t="n"/>
       <c r="D27" s="193" t="inlineStr">
         <is>
-          <t>FINANCIALS + LIST OF SHAREHOLDER</t>
+          <t>PREVIOUS FLA - UNLESS THERE IS CHANGE</t>
         </is>
       </c>
     </row>
@@ -2393,7 +2391,7 @@
       <c r="C28" s="192" t="n"/>
       <c r="D28" s="193" t="inlineStr">
         <is>
-          <t>FINANCIALS + LIST OF SHAREHOLDER</t>
+          <t>PREVIOUS FLA - UNLESS THERE IS CHANGE</t>
         </is>
       </c>
     </row>

</xml_diff>